<commit_message>
Add L2 verification: digit-signature, spread-distribution and source-availability tests
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0168WxZRzFr3YzWSe68Nt1CM
</commit_message>
<xml_diff>
--- a/Smart_Meter_Tenders_L1_L2_VERIFIED.xlsx
+++ b/Smart_Meter_Tenders_L1_L2_VERIFIED.xlsx
@@ -9,7 +9,8 @@
   </bookViews>
   <sheets>
     <sheet name="Audited Bid Data" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Portal Access Status" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="L2 Verification" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Portal Access Status" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -21,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="389" uniqueCount="233">
   <si>
     <t xml:space="preserve">Smart Meter AMISP Tenders — L1/L2 Database, Source-Verified against Primary Documents</t>
   </si>
@@ -288,6 +289,315 @@
   </si>
   <si>
     <t xml:space="preserve">• Genus's real disclosed AMISP LOA values (Aug-2024): ₹2,925.52 cr / ₹3,608.52 cr / ₹4,469.04 cr, for ~3.75 mn and ~5.59 mn meters. Note BSE's own headline metadata mis-states the first as '2,295.52' — the PDF says 2,925.52. None of these match the two Genus rows in your DB.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L2 (Second-Lowest Bidder) — Verification Result</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VERDICT: The L2 column could not be confirmed from ANY public source, and three independent statistical tests indicate the values are modelled rather than observed. The magnitudes are plausible; the numbers are not evidence.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TEST 1 — Digit signature (the decisive one)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Your L1 (₹Cr)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Your L2 (₹Cr)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spread %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L2 rounding</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L1 rounding</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PuVVNL Cluster 1 (Prayagraj &amp; Mirzapur)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">multiple of 10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VERIFIED 2 decimals</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PuVVNL Cluster 2 (Varanasi &amp; Azamgarh)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PuVVNL Cluster 3 (Gorakhpur &amp; Basti)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 decimals</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MVVNL Pkg 1 (Trans Gomti &amp; Bareilly)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">multiple of 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MVVNL Pkg 2 (Lucknow Zone)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MVVNL Pkg 3 (Ayodhya &amp; Devipatan)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DVVNL Pkg 1 (Agra &amp; Aligarh)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DVVNL/KESCo Pkg 2 (Kanpur, Jhansi, Banda)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PVVNL Package (Meerut Zone)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MSEDCL Zone 1 (Bhandup, Kalyan &amp; Konkan)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">round</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MSEDCL Zone 2 (Pune &amp; Baramati)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MSEDCL Zone 3 (Nashik &amp; Jalgaon)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MSEDCL Zone 4 (Latur, Nanded &amp; Aurangabad)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MSEDCL Zone 5 (Nagpur &amp; Amravati)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">APDCL Phase II (Guwahati &amp; Lower Assam)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RESULT: 17 of 17 L2 values are exact multiples of ₹5 cr; 13 of 17 are exact multiples of ₹10 cr.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   By contrast the three L1 values I confirmed against GMR's BSE filings carry real decimals: 2386.72, 2736.65, 2469.71.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Genuine sealed financial bids do not land on round crore figures — they carry paise-level precision like the verified L1s do. A 17-for-17 run of round numbers is not something competitive bidding produces.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TEST 2 — Spread distribution</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metric</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Your data</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What real auctions look like</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L1-L2 spread range</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.07% to 4.63% (1.56 pp wide)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UP tender bids ran +48% to +65% over the REC benchmark — a ~17 pp band</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mean spread</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.72%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No published mean exists; single-tender L1-to-high dispersion reported ~11-13%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Std deviation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.49 pp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Would be several pp across 17 tenders in 4 states over 3+ years</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coefficient of variation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13.3%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bid spreads vary with bidder count, cluster size and state risk — this is far too tight</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Span of the data</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17 packages, 4 states, 2022-2023</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A single narrow band across all of them is a modelling artefact, not a market outcome</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TEST 3 — Source availability (searched exhaustively 21-Aug-2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Source route</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Does it disclose L2?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evidence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BSE/SEBI Reg-30 filings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fetched GMR, Genus, NCC, Adani filings directly. Every one names only the winner and its value. Reg 30 requires disclosure of orders received — never of rival bids.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">News coverage of UP tenders</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Even the adversarial Adani coverage (ThePrint, Business Standard, The Federal, Swarajya, National Herald) reports only L1 per discom: Adani L1 at MVVNL ₹5,400 cr and DVVNL ~₹7,000 cr; GMR L1 at PuVVNL ~₹9,000 cr; IntelliSmart L1 at PVVNL. No L2 anywhere.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prayas (Energy Group) research</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NO — states it is confidential</t>
+  </si>
+  <si>
+    <t xml:space="preserve">'The process of examination, evaluation and comparison of bids is held confidential by utilities along with the information relating to the contract award. AMISPs are also expected to maintain confidentiality of their bids to avoid compromising their competitive positions.'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UPERC tariff orders</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FY27 order (501 pp) mined: gives PMPM ₹101.421 and package-wise rates filed in annexures, but no rival-bid comparison.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GePNIC portals (UP/Maha/Assam)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YES — but CAPTCHA-gated</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AOC / Comparative Statement documents on these portals DO carry the ranked bidder table. Pages load from here; every search requires a CAPTCHA, so they cannot be pulled automatically.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tender aggregators (tenderdetail etc.)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PARTIAL — paywalled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">'15 Awarded Tender Records' for AMISP exist behind a paid 'Competitive Bid Analysis' subscription; no L1/L2 exposed publicly.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WHAT IS REAL AND USABLE FOR COMPETITIVE INTENSITY (all verified)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Source</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REC benchmark rate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">₹6,000 / meter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REC guideline cited across UP tender coverage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adani L1 quote, MVVNL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">₹10,000 / meter (+67% vs benchmark)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ThePrint / The Federal / Swarajya</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reported bid band vs benchmark</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+48% to +65%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Swarajya — the closest thing to a real bid-dispersion figure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Discom meter procurement cost</t>
+  </si>
+  <si>
+    <t xml:space="preserve">₹2,500-2,630 / unit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UP Rajya Vidyut Upbhokta Parishad evidence to UPERC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Consumer charge vs procurement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">₹6,016 charged = +130%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UPERC suo motu order; ~₹200 cr refund to 5+ lakh consumers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RDSS award rates, 33 discoms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">₹7,236-12,118 (median 8,839)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prayas from RDSS dashboard, Apr-2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PMPM service charge won</t>
+  </si>
+  <si>
+    <t xml:space="preserve">₹60 (WB) to ₹167 (MP Paschim)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prayas — a 2.8x spread; the real 'how aggressive was the bid' metric</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Your implied L1 ₹/meter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">₹8,710-12,381 (mean 10,812)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Consistent with the Prayas range — your L1 magnitudes are sensible</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HOW TO GET REAL L2 — the one route that works</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open the state GePNIC portal (etender.up.nic.in / mahatenders.gov.in / assamtenders.gov.in) -&gt; 'Results of Tenders' or 'Tenders in Archive'.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. Search keyword 'AMISP' or 'smart meter' for the relevant discom, solve the CAPTCHA (this is the step I cannot automate).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Open the AOC / 'Comparative Statement' / 'Financial Bid Opening Summary' document — this is where the ranked bidder table with all quoted values sits.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. Send me those PDFs and I will extract every bidder and rate and rebuild this column on observed data, exactly as I did with the GMR filings.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Note: an important structural caveat for the UP rows — three of the four original UP discom tenders were CANCELLED (MVVNL Feb-2023, DVVNL and PuVVNL by Apr-2023) after the pricing controversy, and re-tendered in smaller clusters. Any L1/L2 pair for UP must state whether it belongs to the original or the re-tender; GMR's verified awards are from the RE-TENDER (LOI Jul-2023, LOA Sep-2023).</t>
   </si>
   <si>
     <t xml:space="preserve">Source-Portal Reachability from this environment (tested 21-Aug-2026)</t>
@@ -417,12 +727,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0"/>
     <numFmt numFmtId="166" formatCode="#,##0.00"/>
+    <numFmt numFmtId="167" formatCode="0.00"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -477,6 +788,12 @@
     <font>
       <b val="true"/>
       <sz val="9"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="8.5"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -563,12 +880,16 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="31">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -616,11 +937,51 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -630,6 +991,18 @@
     </xf>
     <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -887,980 +1260,980 @@
   <dimension ref="A1:N31"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="11" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="11" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="12"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
-      <c r="K2" s="2"/>
-      <c r="L2" s="2"/>
-      <c r="M2" s="2"/>
-      <c r="N2" s="2"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
-      <c r="J3" s="2"/>
-      <c r="K3" s="2"/>
-      <c r="L3" s="2"/>
-      <c r="M3" s="2"/>
-      <c r="N3" s="2"/>
-    </row>
-    <row r="5" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
+      <c r="M2" s="3"/>
+      <c r="N2" s="3"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="3"/>
+      <c r="K3" s="3"/>
+      <c r="L3" s="3"/>
+      <c r="M3" s="3"/>
+      <c r="N3" s="3"/>
+    </row>
+    <row r="5" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F5" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="G5" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="H5" s="3" t="s">
+      <c r="H5" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="I5" s="3" t="s">
+      <c r="I5" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="J5" s="3" t="s">
+      <c r="J5" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="K5" s="3" t="s">
+      <c r="K5" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="L5" s="3" t="s">
+      <c r="L5" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="M5" s="3" t="s">
+      <c r="M5" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="N5" s="3" t="s">
+      <c r="N5" s="4" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="5" t="n">
+      <c r="C6" s="6" t="n">
         <v>2520000</v>
       </c>
-      <c r="D6" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="E6" s="4" t="s">
+      <c r="D6" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E6" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="F6" s="4" t="s">
+      <c r="F6" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="G6" s="6" t="n">
+      <c r="G6" s="7" t="n">
         <v>2386.72</v>
       </c>
-      <c r="H6" s="7" t="n">
+      <c r="H6" s="8" t="n">
         <v>2386.72</v>
       </c>
-      <c r="I6" s="4" t="s">
+      <c r="I6" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="J6" s="8" t="n">
+      <c r="J6" s="9" t="n">
         <v>2490</v>
       </c>
-      <c r="K6" s="4" t="s">
+      <c r="K6" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="L6" s="9" t="s">
+      <c r="L6" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="M6" s="4" t="s">
+      <c r="M6" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="N6" s="4" t="s">
+      <c r="N6" s="5" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="C7" s="5" t="n">
+      <c r="C7" s="6" t="n">
         <v>2740000</v>
       </c>
-      <c r="D7" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="E7" s="4" t="s">
+      <c r="D7" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E7" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="F7" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="G7" s="6" t="n">
+      <c r="G7" s="7" t="n">
         <v>2736.66</v>
       </c>
-      <c r="H7" s="7" t="n">
+      <c r="H7" s="8" t="n">
         <v>2736.65</v>
       </c>
-      <c r="I7" s="4" t="s">
+      <c r="I7" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="J7" s="8" t="n">
+      <c r="J7" s="9" t="n">
         <v>2840</v>
       </c>
-      <c r="K7" s="4" t="s">
+      <c r="K7" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="L7" s="9" t="s">
+      <c r="L7" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="M7" s="4" t="s">
+      <c r="M7" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="N7" s="4" t="s">
+      <c r="N7" s="5" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="C8" s="5" t="n">
+      <c r="C8" s="6" t="n">
         <v>2490000</v>
       </c>
-      <c r="D8" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="E8" s="4" t="s">
+      <c r="D8" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E8" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="F8" s="4" t="s">
+      <c r="F8" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="G8" s="6" t="n">
+      <c r="G8" s="7" t="n">
         <v>2666.73</v>
       </c>
-      <c r="H8" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="I8" s="4" t="s">
+      <c r="H8" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="I8" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="J8" s="8" t="n">
+      <c r="J8" s="9" t="n">
         <v>2780</v>
       </c>
-      <c r="K8" s="4" t="s">
+      <c r="K8" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="L8" s="10" t="s">
+      <c r="L8" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="M8" s="4" t="s">
+      <c r="M8" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="N8" s="4" t="s">
+      <c r="N8" s="5" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="C9" s="5" t="n">
+      <c r="C9" s="6" t="n">
         <v>2680000</v>
       </c>
-      <c r="D9" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="E9" s="4" t="s">
+      <c r="D9" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E9" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="F9" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="G9" s="6" t="n">
+      <c r="F9" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="G9" s="7" t="n">
         <v>2934.88</v>
       </c>
-      <c r="H9" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="I9" s="4" t="s">
+      <c r="H9" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="I9" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="J9" s="8" t="n">
+      <c r="J9" s="9" t="n">
         <v>3025</v>
       </c>
-      <c r="K9" s="4" t="s">
+      <c r="K9" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="L9" s="10" t="s">
+      <c r="L9" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="M9" s="4" t="s">
+      <c r="M9" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="N9" s="4" t="s">
+      <c r="N9" s="5" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="C10" s="5" t="n">
+      <c r="C10" s="6" t="n">
         <v>2010000</v>
       </c>
-      <c r="D10" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="E10" s="4" t="s">
+      <c r="D10" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E10" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="F10" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="G10" s="6" t="n">
+      <c r="F10" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="G10" s="7" t="n">
         <v>2138.49</v>
       </c>
-      <c r="H10" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="I10" s="4" t="s">
+      <c r="H10" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="I10" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="J10" s="8" t="n">
+      <c r="J10" s="9" t="n">
         <v>2210</v>
       </c>
-      <c r="K10" s="4" t="s">
+      <c r="K10" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="L10" s="10" t="s">
+      <c r="L10" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="M10" s="4" t="s">
+      <c r="M10" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="N10" s="4" t="s">
+      <c r="N10" s="5" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="C11" s="5" t="n">
+      <c r="C11" s="6" t="n">
         <v>2840000</v>
       </c>
-      <c r="D11" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="E11" s="4" t="s">
+      <c r="D11" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E11" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="F11" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="G11" s="6" t="n">
+      <c r="F11" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="G11" s="7" t="n">
         <v>3073.61</v>
       </c>
-      <c r="H11" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="I11" s="4" t="s">
+      <c r="H11" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="I11" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="J11" s="8" t="n">
+      <c r="J11" s="9" t="n">
         <v>3195</v>
       </c>
-      <c r="K11" s="4" t="s">
+      <c r="K11" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="L11" s="10" t="s">
+      <c r="L11" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="M11" s="4" t="s">
+      <c r="M11" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="N11" s="4" t="s">
+      <c r="N11" s="5" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="s">
+      <c r="A12" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="C12" s="5" t="n">
+      <c r="C12" s="6" t="n">
         <v>2610000</v>
       </c>
-      <c r="D12" s="5" t="n">
+      <c r="D12" s="6" t="n">
         <v>2552000</v>
       </c>
-      <c r="E12" s="4" t="s">
+      <c r="E12" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="F12" s="4" t="s">
+      <c r="F12" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="G12" s="6" t="n">
+      <c r="G12" s="7" t="n">
         <v>2469.71</v>
       </c>
-      <c r="H12" s="7" t="n">
+      <c r="H12" s="8" t="n">
         <v>2469.71</v>
       </c>
-      <c r="I12" s="4" t="s">
+      <c r="I12" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="J12" s="8" t="n">
+      <c r="J12" s="9" t="n">
         <v>2580</v>
       </c>
-      <c r="K12" s="4" t="s">
+      <c r="K12" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="L12" s="9" t="s">
+      <c r="L12" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="M12" s="4" t="s">
+      <c r="M12" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="N12" s="4" t="s">
+      <c r="N12" s="5" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="s">
+      <c r="A13" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="C13" s="5" t="n">
+      <c r="C13" s="6" t="n">
         <v>3560000</v>
       </c>
-      <c r="D13" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="E13" s="4" t="s">
+      <c r="D13" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E13" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="F13" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="G13" s="6" t="n">
+      <c r="F13" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="G13" s="7" t="n">
         <v>3683.27</v>
       </c>
-      <c r="H13" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="I13" s="4" t="s">
+      <c r="H13" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="I13" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="J13" s="8" t="n">
+      <c r="J13" s="9" t="n">
         <v>3810</v>
       </c>
-      <c r="K13" s="4" t="s">
+      <c r="K13" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="L13" s="10" t="s">
+      <c r="L13" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="M13" s="4" t="s">
+      <c r="M13" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="N13" s="4" t="s">
+      <c r="N13" s="5" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="s">
+      <c r="A14" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="C14" s="5" t="n">
+      <c r="C14" s="6" t="n">
         <v>6680000</v>
       </c>
-      <c r="D14" s="5" t="n">
+      <c r="D14" s="6" t="n">
         <v>6684000</v>
       </c>
-      <c r="E14" s="4" t="s">
+      <c r="E14" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="F14" s="4" t="s">
+      <c r="F14" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="G14" s="6" t="n">
+      <c r="G14" s="7" t="n">
         <v>7529.66</v>
       </c>
-      <c r="H14" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="I14" s="4" t="s">
+      <c r="H14" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="I14" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="J14" s="8" t="n">
+      <c r="J14" s="9" t="n">
         <v>7820</v>
       </c>
-      <c r="K14" s="4" t="s">
+      <c r="K14" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="L14" s="10" t="s">
+      <c r="L14" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="M14" s="4" t="s">
+      <c r="M14" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="N14" s="4" t="s">
+      <c r="N14" s="5" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="s">
+      <c r="A15" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="C15" s="5" t="n">
+      <c r="C15" s="6" t="n">
         <v>6344000</v>
       </c>
-      <c r="D15" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="E15" s="4" t="s">
+      <c r="D15" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E15" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="F15" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="G15" s="6" t="n">
+      <c r="F15" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="G15" s="7" t="n">
         <v>7525</v>
       </c>
-      <c r="H15" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="I15" s="4" t="s">
+      <c r="H15" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="I15" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="J15" s="8" t="n">
+      <c r="J15" s="9" t="n">
         <v>7760</v>
       </c>
-      <c r="K15" s="4" t="s">
+      <c r="K15" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="L15" s="10" t="s">
+      <c r="L15" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="M15" s="4" t="s">
+      <c r="M15" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="N15" s="4" t="s">
+      <c r="N15" s="5" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="s">
+      <c r="A16" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="C16" s="5" t="n">
+      <c r="C16" s="6" t="n">
         <v>5245000</v>
       </c>
-      <c r="D16" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="E16" s="4" t="s">
+      <c r="D16" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E16" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="F16" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="G16" s="6" t="n">
+      <c r="F16" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="G16" s="7" t="n">
         <v>6388</v>
       </c>
-      <c r="H16" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="I16" s="4" t="s">
+      <c r="H16" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="I16" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="J16" s="8" t="n">
+      <c r="J16" s="9" t="n">
         <v>6590</v>
       </c>
-      <c r="K16" s="4" t="s">
+      <c r="K16" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="L16" s="10" t="s">
+      <c r="L16" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="M16" s="4" t="s">
+      <c r="M16" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="N16" s="4" t="s">
+      <c r="N16" s="5" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
+      <c r="A17" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="C17" s="5" t="n">
+      <c r="C17" s="6" t="n">
         <v>2886000</v>
       </c>
-      <c r="D17" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="E17" s="4" t="s">
+      <c r="D17" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E17" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="F17" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="G17" s="6" t="n">
+      <c r="F17" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="G17" s="7" t="n">
         <v>3461</v>
       </c>
-      <c r="H17" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="I17" s="4" t="s">
+      <c r="H17" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="I17" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="J17" s="8" t="n">
+      <c r="J17" s="9" t="n">
         <v>3570</v>
       </c>
-      <c r="K17" s="4" t="s">
+      <c r="K17" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="L17" s="11" t="s">
+      <c r="L17" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="M17" s="4" t="s">
+      <c r="M17" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="N17" s="4" t="s">
+      <c r="N17" s="5" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4" t="s">
+      <c r="A18" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="B18" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="C18" s="5" t="n">
+      <c r="C18" s="6" t="n">
         <v>2777000</v>
       </c>
-      <c r="D18" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="E18" s="4" t="s">
+      <c r="D18" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E18" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="F18" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="G18" s="6" t="n">
+      <c r="F18" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="G18" s="7" t="n">
         <v>3330</v>
       </c>
-      <c r="H18" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="I18" s="4" t="s">
+      <c r="H18" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="I18" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="J18" s="8" t="n">
+      <c r="J18" s="9" t="n">
         <v>3445</v>
       </c>
-      <c r="K18" s="4" t="s">
+      <c r="K18" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="L18" s="11" t="s">
+      <c r="L18" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="M18" s="4" t="s">
+      <c r="M18" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="N18" s="4" t="s">
+      <c r="N18" s="5" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4" t="s">
+      <c r="A19" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="B19" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="C19" s="5" t="n">
+      <c r="C19" s="6" t="n">
         <v>3110000</v>
       </c>
-      <c r="D19" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="E19" s="4" t="s">
+      <c r="D19" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E19" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="F19" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="G19" s="6" t="n">
+      <c r="F19" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="G19" s="7" t="n">
         <v>3710</v>
       </c>
-      <c r="H19" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="I19" s="4" t="s">
+      <c r="H19" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="I19" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="J19" s="8" t="n">
+      <c r="J19" s="9" t="n">
         <v>3840</v>
       </c>
-      <c r="K19" s="4" t="s">
+      <c r="K19" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="L19" s="10" t="s">
+      <c r="L19" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="M19" s="4" t="s">
+      <c r="M19" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="N19" s="4" t="s">
+      <c r="N19" s="5" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4" t="s">
+      <c r="A20" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="B20" s="4" t="s">
+      <c r="B20" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="C20" s="5" t="n">
+      <c r="C20" s="6" t="n">
         <v>1050000</v>
       </c>
-      <c r="D20" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="E20" s="4" t="s">
+      <c r="D20" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E20" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="F20" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="G20" s="6" t="n">
+      <c r="F20" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="G20" s="7" t="n">
         <v>1300</v>
       </c>
-      <c r="H20" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="I20" s="4" t="s">
+      <c r="H20" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="I20" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="J20" s="8" t="n">
+      <c r="J20" s="9" t="n">
         <v>1350</v>
       </c>
-      <c r="K20" s="4" t="s">
+      <c r="K20" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="L20" s="10" t="s">
+      <c r="L20" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="M20" s="4" t="s">
+      <c r="M20" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="N20" s="4" t="s">
+      <c r="N20" s="5" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4" t="s">
+      <c r="A21" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="B21" s="4" t="s">
+      <c r="B21" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="C21" s="5" t="n">
+      <c r="C21" s="6" t="n">
         <v>7040000</v>
       </c>
-      <c r="D21" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="E21" s="4" t="s">
+      <c r="D21" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E21" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="F21" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="G21" s="6" t="n">
+      <c r="F21" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="G21" s="7" t="n">
         <v>6400</v>
       </c>
-      <c r="H21" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="I21" s="4" t="s">
+      <c r="H21" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="I21" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="J21" s="8" t="n">
+      <c r="J21" s="9" t="n">
         <v>6650</v>
       </c>
-      <c r="K21" s="4" t="s">
+      <c r="K21" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="L21" s="10" t="s">
+      <c r="L21" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="M21" s="4" t="s">
+      <c r="M21" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="N21" s="4" t="s">
+      <c r="N21" s="5" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4" t="s">
+      <c r="A22" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="B22" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="C22" s="5" t="n">
+      <c r="C22" s="6" t="n">
         <v>620000</v>
       </c>
-      <c r="D22" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="E22" s="4" t="s">
+      <c r="D22" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E22" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="F22" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="G22" s="6" t="n">
+      <c r="F22" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="G22" s="7" t="n">
         <v>540</v>
       </c>
-      <c r="H22" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="I22" s="4" t="s">
+      <c r="H22" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="I22" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="J22" s="8" t="n">
+      <c r="J22" s="9" t="n">
         <v>565</v>
       </c>
-      <c r="K22" s="4" t="s">
+      <c r="K22" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="L22" s="10" t="s">
+      <c r="L22" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="M22" s="4" t="s">
+      <c r="M22" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="N22" s="4" t="s">
+      <c r="N22" s="5" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="1" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="2" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="12" t="s">
+      <c r="A25" s="13" t="s">
         <v>82</v>
       </c>
-      <c r="B25" s="12"/>
-      <c r="C25" s="12"/>
-      <c r="D25" s="12"/>
-      <c r="E25" s="12"/>
-      <c r="F25" s="12"/>
-      <c r="G25" s="12"/>
-      <c r="H25" s="12"/>
-      <c r="I25" s="12"/>
-      <c r="J25" s="12"/>
-      <c r="K25" s="12"/>
-      <c r="L25" s="12"/>
-      <c r="M25" s="12"/>
-      <c r="N25" s="12"/>
+      <c r="B25" s="13"/>
+      <c r="C25" s="13"/>
+      <c r="D25" s="13"/>
+      <c r="E25" s="13"/>
+      <c r="F25" s="13"/>
+      <c r="G25" s="13"/>
+      <c r="H25" s="13"/>
+      <c r="I25" s="13"/>
+      <c r="J25" s="13"/>
+      <c r="K25" s="13"/>
+      <c r="L25" s="13"/>
+      <c r="M25" s="13"/>
+      <c r="N25" s="13"/>
     </row>
     <row r="26" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="12" t="s">
+      <c r="A26" s="13" t="s">
         <v>83</v>
       </c>
-      <c r="B26" s="12"/>
-      <c r="C26" s="12"/>
-      <c r="D26" s="12"/>
-      <c r="E26" s="12"/>
-      <c r="F26" s="12"/>
-      <c r="G26" s="12"/>
-      <c r="H26" s="12"/>
-      <c r="I26" s="12"/>
-      <c r="J26" s="12"/>
-      <c r="K26" s="12"/>
-      <c r="L26" s="12"/>
-      <c r="M26" s="12"/>
-      <c r="N26" s="12"/>
+      <c r="B26" s="13"/>
+      <c r="C26" s="13"/>
+      <c r="D26" s="13"/>
+      <c r="E26" s="13"/>
+      <c r="F26" s="13"/>
+      <c r="G26" s="13"/>
+      <c r="H26" s="13"/>
+      <c r="I26" s="13"/>
+      <c r="J26" s="13"/>
+      <c r="K26" s="13"/>
+      <c r="L26" s="13"/>
+      <c r="M26" s="13"/>
+      <c r="N26" s="13"/>
     </row>
     <row r="27" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="12" t="s">
+      <c r="A27" s="13" t="s">
         <v>84</v>
       </c>
-      <c r="B27" s="12"/>
-      <c r="C27" s="12"/>
-      <c r="D27" s="12"/>
-      <c r="E27" s="12"/>
-      <c r="F27" s="12"/>
-      <c r="G27" s="12"/>
-      <c r="H27" s="12"/>
-      <c r="I27" s="12"/>
-      <c r="J27" s="12"/>
-      <c r="K27" s="12"/>
-      <c r="L27" s="12"/>
-      <c r="M27" s="12"/>
-      <c r="N27" s="12"/>
+      <c r="B27" s="13"/>
+      <c r="C27" s="13"/>
+      <c r="D27" s="13"/>
+      <c r="E27" s="13"/>
+      <c r="F27" s="13"/>
+      <c r="G27" s="13"/>
+      <c r="H27" s="13"/>
+      <c r="I27" s="13"/>
+      <c r="J27" s="13"/>
+      <c r="K27" s="13"/>
+      <c r="L27" s="13"/>
+      <c r="M27" s="13"/>
+      <c r="N27" s="13"/>
     </row>
     <row r="28" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="12" t="s">
+      <c r="A28" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="B28" s="12"/>
-      <c r="C28" s="12"/>
-      <c r="D28" s="12"/>
-      <c r="E28" s="12"/>
-      <c r="F28" s="12"/>
-      <c r="G28" s="12"/>
-      <c r="H28" s="12"/>
-      <c r="I28" s="12"/>
-      <c r="J28" s="12"/>
-      <c r="K28" s="12"/>
-      <c r="L28" s="12"/>
-      <c r="M28" s="12"/>
-      <c r="N28" s="12"/>
+      <c r="B28" s="13"/>
+      <c r="C28" s="13"/>
+      <c r="D28" s="13"/>
+      <c r="E28" s="13"/>
+      <c r="F28" s="13"/>
+      <c r="G28" s="13"/>
+      <c r="H28" s="13"/>
+      <c r="I28" s="13"/>
+      <c r="J28" s="13"/>
+      <c r="K28" s="13"/>
+      <c r="L28" s="13"/>
+      <c r="M28" s="13"/>
+      <c r="N28" s="13"/>
     </row>
     <row r="29" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="12" t="s">
+      <c r="A29" s="13" t="s">
         <v>86</v>
       </c>
-      <c r="B29" s="12"/>
-      <c r="C29" s="12"/>
-      <c r="D29" s="12"/>
-      <c r="E29" s="12"/>
-      <c r="F29" s="12"/>
-      <c r="G29" s="12"/>
-      <c r="H29" s="12"/>
-      <c r="I29" s="12"/>
-      <c r="J29" s="12"/>
-      <c r="K29" s="12"/>
-      <c r="L29" s="12"/>
-      <c r="M29" s="12"/>
-      <c r="N29" s="12"/>
+      <c r="B29" s="13"/>
+      <c r="C29" s="13"/>
+      <c r="D29" s="13"/>
+      <c r="E29" s="13"/>
+      <c r="F29" s="13"/>
+      <c r="G29" s="13"/>
+      <c r="H29" s="13"/>
+      <c r="I29" s="13"/>
+      <c r="J29" s="13"/>
+      <c r="K29" s="13"/>
+      <c r="L29" s="13"/>
+      <c r="M29" s="13"/>
+      <c r="N29" s="13"/>
     </row>
     <row r="30" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="12" t="s">
+      <c r="A30" s="13" t="s">
         <v>87</v>
       </c>
-      <c r="B30" s="12"/>
-      <c r="C30" s="12"/>
-      <c r="D30" s="12"/>
-      <c r="E30" s="12"/>
-      <c r="F30" s="12"/>
-      <c r="G30" s="12"/>
-      <c r="H30" s="12"/>
-      <c r="I30" s="12"/>
-      <c r="J30" s="12"/>
-      <c r="K30" s="12"/>
-      <c r="L30" s="12"/>
-      <c r="M30" s="12"/>
-      <c r="N30" s="12"/>
+      <c r="B30" s="13"/>
+      <c r="C30" s="13"/>
+      <c r="D30" s="13"/>
+      <c r="E30" s="13"/>
+      <c r="F30" s="13"/>
+      <c r="G30" s="13"/>
+      <c r="H30" s="13"/>
+      <c r="I30" s="13"/>
+      <c r="J30" s="13"/>
+      <c r="K30" s="13"/>
+      <c r="L30" s="13"/>
+      <c r="M30" s="13"/>
+      <c r="N30" s="13"/>
     </row>
     <row r="31" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="12" t="s">
+      <c r="A31" s="13" t="s">
         <v>88</v>
       </c>
-      <c r="B31" s="12"/>
-      <c r="C31" s="12"/>
-      <c r="D31" s="12"/>
-      <c r="E31" s="12"/>
-      <c r="F31" s="12"/>
-      <c r="G31" s="12"/>
-      <c r="H31" s="12"/>
-      <c r="I31" s="12"/>
-      <c r="J31" s="12"/>
-      <c r="K31" s="12"/>
-      <c r="L31" s="12"/>
-      <c r="M31" s="12"/>
-      <c r="N31" s="12"/>
+      <c r="B31" s="13"/>
+      <c r="C31" s="13"/>
+      <c r="D31" s="13"/>
+      <c r="E31" s="13"/>
+      <c r="F31" s="13"/>
+      <c r="G31" s="13"/>
+      <c r="H31" s="13"/>
+      <c r="I31" s="13"/>
+      <c r="J31" s="13"/>
+      <c r="K31" s="13"/>
+      <c r="L31" s="13"/>
+      <c r="M31" s="13"/>
+      <c r="N31" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -1888,172 +2261,939 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:H61"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="14" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="15" t="s">
+        <v>90</v>
+      </c>
+      <c r="B2" s="15"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
+      <c r="G2" s="15"/>
+      <c r="H2" s="15"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="15"/>
+      <c r="B3" s="15"/>
+      <c r="C3" s="15"/>
+      <c r="D3" s="15"/>
+      <c r="E3" s="15"/>
+      <c r="F3" s="15"/>
+      <c r="G3" s="15"/>
+      <c r="H3" s="15"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="16" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="17" t="s">
+        <v>92</v>
+      </c>
+      <c r="C6" s="17" t="s">
+        <v>93</v>
+      </c>
+      <c r="D6" s="17" t="s">
+        <v>94</v>
+      </c>
+      <c r="E6" s="17" t="s">
+        <v>95</v>
+      </c>
+      <c r="F6" s="17" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="18" t="s">
+        <v>97</v>
+      </c>
+      <c r="B7" s="19" t="n">
+        <v>2386.72</v>
+      </c>
+      <c r="C7" s="19" t="n">
+        <v>2490</v>
+      </c>
+      <c r="D7" s="20" t="n">
+        <v>4.33</v>
+      </c>
+      <c r="E7" s="21" t="s">
+        <v>98</v>
+      </c>
+      <c r="F7" s="22" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="18" t="s">
+        <v>100</v>
+      </c>
+      <c r="B8" s="19" t="n">
+        <v>2736.66</v>
+      </c>
+      <c r="C8" s="19" t="n">
+        <v>2840</v>
+      </c>
+      <c r="D8" s="20" t="n">
+        <v>3.78</v>
+      </c>
+      <c r="E8" s="21" t="s">
+        <v>98</v>
+      </c>
+      <c r="F8" s="22" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="18" t="s">
+        <v>101</v>
+      </c>
+      <c r="B9" s="19" t="n">
+        <v>2666.73</v>
+      </c>
+      <c r="C9" s="19" t="n">
+        <v>2780</v>
+      </c>
+      <c r="D9" s="20" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="E9" s="21" t="s">
+        <v>98</v>
+      </c>
+      <c r="F9" s="18" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="18" t="s">
+        <v>103</v>
+      </c>
+      <c r="B10" s="19" t="n">
+        <v>2934.88</v>
+      </c>
+      <c r="C10" s="19" t="n">
+        <v>3025</v>
+      </c>
+      <c r="D10" s="20" t="n">
+        <v>3.07</v>
+      </c>
+      <c r="E10" s="21" t="s">
+        <v>104</v>
+      </c>
+      <c r="F10" s="18" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="18" t="s">
+        <v>105</v>
+      </c>
+      <c r="B11" s="19" t="n">
+        <v>2138.49</v>
+      </c>
+      <c r="C11" s="19" t="n">
+        <v>2210</v>
+      </c>
+      <c r="D11" s="20" t="n">
+        <v>3.34</v>
+      </c>
+      <c r="E11" s="21" t="s">
+        <v>98</v>
+      </c>
+      <c r="F11" s="18" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="18" t="s">
+        <v>106</v>
+      </c>
+      <c r="B12" s="19" t="n">
+        <v>3073.61</v>
+      </c>
+      <c r="C12" s="19" t="n">
+        <v>3195</v>
+      </c>
+      <c r="D12" s="20" t="n">
+        <v>3.95</v>
+      </c>
+      <c r="E12" s="21" t="s">
+        <v>104</v>
+      </c>
+      <c r="F12" s="18" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="B13" s="19" t="n">
+        <v>2469.71</v>
+      </c>
+      <c r="C13" s="19" t="n">
+        <v>2580</v>
+      </c>
+      <c r="D13" s="20" t="n">
+        <v>4.47</v>
+      </c>
+      <c r="E13" s="21" t="s">
+        <v>98</v>
+      </c>
+      <c r="F13" s="22" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="18" t="s">
+        <v>108</v>
+      </c>
+      <c r="B14" s="19" t="n">
+        <v>3683.27</v>
+      </c>
+      <c r="C14" s="19" t="n">
+        <v>3810</v>
+      </c>
+      <c r="D14" s="20" t="n">
+        <v>3.44</v>
+      </c>
+      <c r="E14" s="21" t="s">
+        <v>98</v>
+      </c>
+      <c r="F14" s="18" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="18" t="s">
+        <v>109</v>
+      </c>
+      <c r="B15" s="19" t="n">
+        <v>7529.66</v>
+      </c>
+      <c r="C15" s="19" t="n">
+        <v>7820</v>
+      </c>
+      <c r="D15" s="20" t="n">
+        <v>3.86</v>
+      </c>
+      <c r="E15" s="21" t="s">
+        <v>98</v>
+      </c>
+      <c r="F15" s="18" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="18" t="s">
+        <v>110</v>
+      </c>
+      <c r="B16" s="19" t="n">
+        <v>7525</v>
+      </c>
+      <c r="C16" s="19" t="n">
+        <v>7760</v>
+      </c>
+      <c r="D16" s="20" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="E16" s="21" t="s">
+        <v>98</v>
+      </c>
+      <c r="F16" s="18" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="18" t="s">
+        <v>112</v>
+      </c>
+      <c r="B17" s="19" t="n">
+        <v>6388</v>
+      </c>
+      <c r="C17" s="19" t="n">
+        <v>6590</v>
+      </c>
+      <c r="D17" s="20" t="n">
+        <v>3.16</v>
+      </c>
+      <c r="E17" s="21" t="s">
+        <v>98</v>
+      </c>
+      <c r="F17" s="18" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="18" t="s">
+        <v>113</v>
+      </c>
+      <c r="B18" s="19" t="n">
+        <v>3461</v>
+      </c>
+      <c r="C18" s="19" t="n">
+        <v>3570</v>
+      </c>
+      <c r="D18" s="20" t="n">
+        <v>3.15</v>
+      </c>
+      <c r="E18" s="21" t="s">
+        <v>98</v>
+      </c>
+      <c r="F18" s="18" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="B19" s="19" t="n">
+        <v>3330</v>
+      </c>
+      <c r="C19" s="19" t="n">
+        <v>3445</v>
+      </c>
+      <c r="D19" s="20" t="n">
+        <v>3.45</v>
+      </c>
+      <c r="E19" s="21" t="s">
+        <v>104</v>
+      </c>
+      <c r="F19" s="18" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="18" t="s">
+        <v>115</v>
+      </c>
+      <c r="B20" s="19" t="n">
+        <v>3710</v>
+      </c>
+      <c r="C20" s="19" t="n">
+        <v>3840</v>
+      </c>
+      <c r="D20" s="20" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="E20" s="21" t="s">
+        <v>98</v>
+      </c>
+      <c r="F20" s="18" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="B21" s="19" t="n">
+        <v>1300</v>
+      </c>
+      <c r="C21" s="19" t="n">
+        <v>1350</v>
+      </c>
+      <c r="D21" s="20" t="n">
+        <v>3.85</v>
+      </c>
+      <c r="E21" s="21" t="s">
+        <v>98</v>
+      </c>
+      <c r="F21" s="18" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="18" t="s">
+        <v>75</v>
+      </c>
+      <c r="B22" s="19" t="n">
+        <v>6400</v>
+      </c>
+      <c r="C22" s="19" t="n">
+        <v>6650</v>
+      </c>
+      <c r="D22" s="20" t="n">
+        <v>3.91</v>
+      </c>
+      <c r="E22" s="21" t="s">
+        <v>98</v>
+      </c>
+      <c r="F22" s="18" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="18" t="s">
+        <v>116</v>
+      </c>
+      <c r="B23" s="19" t="n">
+        <v>540</v>
+      </c>
+      <c r="C23" s="19" t="n">
+        <v>565</v>
+      </c>
+      <c r="D23" s="20" t="n">
+        <v>4.63</v>
+      </c>
+      <c r="E23" s="21" t="s">
+        <v>104</v>
+      </c>
+      <c r="F23" s="18" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="23" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="24" t="s">
+        <v>118</v>
+      </c>
+      <c r="B25" s="24"/>
+      <c r="C25" s="24"/>
+      <c r="D25" s="24"/>
+      <c r="E25" s="24"/>
+      <c r="F25" s="24"/>
+    </row>
+    <row r="26" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="24" t="s">
+        <v>119</v>
+      </c>
+      <c r="B26" s="24"/>
+      <c r="C26" s="24"/>
+      <c r="D26" s="24"/>
+      <c r="E26" s="24"/>
+      <c r="F26" s="24"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="16" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="17" t="s">
+        <v>121</v>
+      </c>
+      <c r="B29" s="17" t="s">
+        <v>122</v>
+      </c>
+      <c r="C29" s="17" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="25" t="s">
+        <v>124</v>
+      </c>
+      <c r="B30" s="26" t="s">
+        <v>125</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="25" t="s">
+        <v>127</v>
+      </c>
+      <c r="B31" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="25" t="s">
+        <v>130</v>
+      </c>
+      <c r="B32" s="26" t="s">
+        <v>131</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="25" t="s">
+        <v>133</v>
+      </c>
+      <c r="B33" s="26" t="s">
+        <v>134</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="25" t="s">
+        <v>136</v>
+      </c>
+      <c r="B34" s="26" t="s">
+        <v>137</v>
+      </c>
+      <c r="C34" s="5" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="16" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="17" t="s">
+        <v>140</v>
+      </c>
+      <c r="B37" s="17" t="s">
+        <v>141</v>
+      </c>
+      <c r="C37" s="17" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="25" t="s">
+        <v>143</v>
+      </c>
+      <c r="B38" s="27" t="s">
+        <v>144</v>
+      </c>
+      <c r="C38" s="5" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="25" t="s">
+        <v>146</v>
+      </c>
+      <c r="B39" s="27" t="s">
+        <v>144</v>
+      </c>
+      <c r="C39" s="5" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="25" t="s">
+        <v>148</v>
+      </c>
+      <c r="B40" s="27" t="s">
+        <v>149</v>
+      </c>
+      <c r="C40" s="5" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="25" t="s">
+        <v>151</v>
+      </c>
+      <c r="B41" s="27" t="s">
+        <v>144</v>
+      </c>
+      <c r="C41" s="5" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="25" t="s">
+        <v>153</v>
+      </c>
+      <c r="B42" s="28" t="s">
+        <v>154</v>
+      </c>
+      <c r="C42" s="5" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="25" t="s">
+        <v>156</v>
+      </c>
+      <c r="B43" s="26" t="s">
+        <v>157</v>
+      </c>
+      <c r="C43" s="5" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="16" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="17" t="s">
+        <v>121</v>
+      </c>
+      <c r="B46" s="17" t="s">
+        <v>160</v>
+      </c>
+      <c r="C46" s="17" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="25" t="s">
+        <v>162</v>
+      </c>
+      <c r="B47" s="28" t="s">
+        <v>163</v>
+      </c>
+      <c r="C47" s="5" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="25" t="s">
+        <v>165</v>
+      </c>
+      <c r="B48" s="28" t="s">
+        <v>166</v>
+      </c>
+      <c r="C48" s="5" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="25" t="s">
+        <v>168</v>
+      </c>
+      <c r="B49" s="28" t="s">
+        <v>169</v>
+      </c>
+      <c r="C49" s="5" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="25" t="s">
+        <v>171</v>
+      </c>
+      <c r="B50" s="28" t="s">
+        <v>172</v>
+      </c>
+      <c r="C50" s="5" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="25" t="s">
+        <v>174</v>
+      </c>
+      <c r="B51" s="28" t="s">
+        <v>175</v>
+      </c>
+      <c r="C51" s="5" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="25" t="s">
+        <v>177</v>
+      </c>
+      <c r="B52" s="28" t="s">
+        <v>178</v>
+      </c>
+      <c r="C52" s="5" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="25" t="s">
+        <v>180</v>
+      </c>
+      <c r="B53" s="28" t="s">
+        <v>181</v>
+      </c>
+      <c r="C53" s="5" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A54" s="25" t="s">
+        <v>183</v>
+      </c>
+      <c r="B54" s="28" t="s">
+        <v>184</v>
+      </c>
+      <c r="C54" s="5" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="16" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A57" s="29" t="s">
+        <v>187</v>
+      </c>
+      <c r="B57" s="29"/>
+      <c r="C57" s="29"/>
+      <c r="D57" s="29"/>
+      <c r="E57" s="29"/>
+      <c r="F57" s="29"/>
+    </row>
+    <row r="58" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A58" s="29" t="s">
+        <v>188</v>
+      </c>
+      <c r="B58" s="29"/>
+      <c r="C58" s="29"/>
+      <c r="D58" s="29"/>
+      <c r="E58" s="29"/>
+      <c r="F58" s="29"/>
+    </row>
+    <row r="59" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A59" s="29" t="s">
+        <v>189</v>
+      </c>
+      <c r="B59" s="29"/>
+      <c r="C59" s="29"/>
+      <c r="D59" s="29"/>
+      <c r="E59" s="29"/>
+      <c r="F59" s="29"/>
+    </row>
+    <row r="60" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A60" s="29" t="s">
+        <v>190</v>
+      </c>
+      <c r="B60" s="29"/>
+      <c r="C60" s="29"/>
+      <c r="D60" s="29"/>
+      <c r="E60" s="29"/>
+      <c r="F60" s="29"/>
+    </row>
+    <row r="61" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A61" s="29" t="s">
+        <v>191</v>
+      </c>
+      <c r="B61" s="29"/>
+      <c r="C61" s="29"/>
+      <c r="D61" s="29"/>
+      <c r="E61" s="29"/>
+      <c r="F61" s="29"/>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="A2:H3"/>
+    <mergeCell ref="A25:F25"/>
+    <mergeCell ref="A26:F26"/>
+    <mergeCell ref="A57:F57"/>
+    <mergeCell ref="A58:F58"/>
+    <mergeCell ref="A59:F59"/>
+    <mergeCell ref="A60:F60"/>
+    <mergeCell ref="A61:F61"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:D13"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="72"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="13" t="s">
-        <v>90</v>
-      </c>
-      <c r="B3" s="13" t="s">
-        <v>91</v>
-      </c>
-      <c r="C3" s="13" t="s">
-        <v>92</v>
-      </c>
-      <c r="D3" s="13" t="s">
-        <v>93</v>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="30" t="s">
+        <v>193</v>
+      </c>
+      <c r="B3" s="30" t="s">
+        <v>194</v>
+      </c>
+      <c r="C3" s="30" t="s">
+        <v>195</v>
+      </c>
+      <c r="D3" s="30" t="s">
+        <v>196</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="C4" s="14" t="s">
-        <v>96</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>97</v>
+      <c r="A4" s="5" t="s">
+        <v>197</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>198</v>
+      </c>
+      <c r="C4" s="28" t="s">
+        <v>199</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>200</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="C5" s="15" t="s">
-        <v>100</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>101</v>
+      <c r="A5" s="5" t="s">
+        <v>201</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="C5" s="26" t="s">
+        <v>203</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>204</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="C6" s="15" t="s">
-        <v>100</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>104</v>
+      <c r="A6" s="5" t="s">
+        <v>205</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>206</v>
+      </c>
+      <c r="C6" s="26" t="s">
+        <v>203</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="C7" s="14" t="s">
-        <v>107</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>108</v>
+      <c r="A7" s="5" t="s">
+        <v>208</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>209</v>
+      </c>
+      <c r="C7" s="28" t="s">
+        <v>210</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>211</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="C8" s="15" t="s">
-        <v>100</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>111</v>
+      <c r="A8" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>213</v>
+      </c>
+      <c r="C8" s="26" t="s">
+        <v>203</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>214</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="C9" s="16" t="s">
-        <v>114</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>115</v>
+      <c r="A9" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="C9" s="27" t="s">
+        <v>217</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>218</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>117</v>
-      </c>
-      <c r="C10" s="15" t="s">
-        <v>118</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>119</v>
+      <c r="A10" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>220</v>
+      </c>
+      <c r="C10" s="26" t="s">
+        <v>221</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>222</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>121</v>
-      </c>
-      <c r="C11" s="14" t="s">
-        <v>96</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>122</v>
+      <c r="A11" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>224</v>
+      </c>
+      <c r="C11" s="28" t="s">
+        <v>199</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>225</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="s">
-        <v>123</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>124</v>
-      </c>
-      <c r="C12" s="16" t="s">
-        <v>125</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>126</v>
+      <c r="A12" s="5" t="s">
+        <v>226</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>227</v>
+      </c>
+      <c r="C12" s="27" t="s">
+        <v>228</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>229</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>128</v>
-      </c>
-      <c r="C13" s="14" t="s">
-        <v>96</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>129</v>
+      <c r="A13" s="5" t="s">
+        <v>230</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="C13" s="28" t="s">
+        <v>199</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>232</v>
       </c>
     </row>
   </sheetData>

</xml_diff>